<commit_message>
Corregir rango: mínimo = cantidades establecidas, máximo hacia arriba
El mínimo es el compromiso del dashboard; el máximo permite usar
tela adicional sin sobrestock (tope +15% o 6 meses cobertura).

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SHORT_PLAYA_SUBL_RANGO_PRODUCCION.xlsx
+++ b/SHORT_PLAYA_SUBL_RANGO_PRODUCCION.xlsx
@@ -40,7 +40,7 @@
       <sz val="13"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -55,11 +55,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00A8D5A2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E3F2FD"/>
       </patternFill>
     </fill>
     <fill>
@@ -114,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,9 +129,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -145,16 +137,13 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -523,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -615,17 +604,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Mínimo</t>
+          <t>Mínimo (compromiso)</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Solicitado (dashboard)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Máximo</t>
+          <t>Máximo (con tela adicional)</t>
         </is>
       </c>
     </row>
@@ -636,13 +620,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>269</v>
+        <v>311</v>
       </c>
       <c r="C11" t="n">
-        <v>311</v>
-      </c>
-      <c r="D11" t="n">
-        <v>343</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12">
@@ -652,13 +633,10 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="C12" t="n">
-        <v>70</v>
-      </c>
-      <c r="D12" t="n">
-        <v>76</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13">
@@ -668,13 +646,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>327</v>
+        <v>381</v>
       </c>
       <c r="C13" t="n">
-        <v>381</v>
-      </c>
-      <c r="D13" t="n">
-        <v>419</v>
+        <v>446</v>
       </c>
     </row>
     <row r="15">
@@ -687,28 +662,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>• Solicitado = cantidades del dashboard (curva óptima, cobertura 3 meses, temporada alta).</t>
+          <t>• Mínimo = cantidades establecidas en el dashboard (compromiso de producción).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>• Mínimo = piso operativo para no quedar cortos en tallas núcleo.</t>
+          <t>• Máximo = techo si hay tela disponible (hasta +15% o 6 meses cobertura, lo que sea menor).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>• Máximo = tope anti-sobrestock (menor entre +10% y 6 meses de cobertura por talla).</t>
+          <t>• La diferencia entre Mín y Máx es el rango de acción hacia arriba.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>• Incluye color de lanzamiento y proyección de red ampliada (VELA, Barquisimeto).</t>
+          <t>• Incluye color de lanzamiento y proyección temporada alta / tiendas nuevas.</t>
         </is>
       </c>
     </row>
@@ -723,31 +698,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>CANTIDADES POR COLORES — RANGO DE ACCIÓN</t>
+          <t>CANTIDADES POR COLORES — MÍNIMO Y MÁXIMO</t>
         </is>
       </c>
     </row>
@@ -762,22 +732,22 @@
           <t>S</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
           <t>XL</t>
         </is>
       </c>
-      <c r="N2" s="5" t="inlineStr">
+      <c r="J2" s="5" t="inlineStr">
         <is>
           <t>2XL</t>
         </is>
@@ -791,29 +761,29 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
@@ -821,269 +791,186 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="N3" s="6" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="O3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Playuela</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="12" t="n"/>
-      <c r="E4" s="13" t="n">
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="11" t="n">
+        <v>26</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>28</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Sal</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="11" t="n">
+        <v>15</v>
+      </c>
+      <c r="E5" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>32</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>37</v>
+      </c>
+      <c r="H5" s="11" t="n">
+        <v>21</v>
+      </c>
+      <c r="I5" s="11" t="n">
+        <v>24</v>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Tucupido</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="E6" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Sombrero</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Nuevo color (lanzamiento)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
+        <v>17</v>
+      </c>
+      <c r="C8" s="11" t="n">
+        <v>20</v>
+      </c>
+      <c r="D8" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>41</v>
+      </c>
+      <c r="G8" s="11" t="n">
+        <v>49</v>
+      </c>
+      <c r="H8" s="11" t="n">
+        <v>29</v>
+      </c>
+      <c r="I8" s="11" t="n">
+        <v>35</v>
+      </c>
+      <c r="J8" s="11" t="n">
+        <v>19</v>
+      </c>
+      <c r="K8" s="11" t="n">
         <v>23</v>
       </c>
-      <c r="F4" s="13" t="n">
-        <v>26</v>
-      </c>
-      <c r="G4" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="H4" s="13" t="n">
-        <v>25</v>
-      </c>
-      <c r="I4" s="13" t="n">
-        <v>28</v>
-      </c>
-      <c r="J4" s="13" t="n">
-        <v>31</v>
-      </c>
-      <c r="K4" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="L4" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="M4" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="N4" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="P4" s="13" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Sal</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="F5" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="G5" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="H5" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="J5" s="13" t="n">
-        <v>35</v>
-      </c>
-      <c r="K5" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="L5" s="13" t="n">
-        <v>21</v>
-      </c>
-      <c r="M5" s="13" t="n">
-        <v>23</v>
-      </c>
-      <c r="N5" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="O5" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="P5" s="13" t="n">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Tucupido</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="F6" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="G6" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="H6" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="I6" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="J6" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="10" t="n"/>
-      <c r="O6" s="11" t="n"/>
-      <c r="P6" s="12" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Sombrero</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="11" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="11" t="n"/>
-      <c r="P7" s="12" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Nuevo color (lanzamiento)</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="C8" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="E8" s="13" t="n">
-        <v>37</v>
-      </c>
-      <c r="F8" s="13" t="n">
-        <v>41</v>
-      </c>
-      <c r="G8" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="H8" s="13" t="n">
-        <v>37</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>41</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>45</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>26</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>29</v>
-      </c>
-      <c r="M8" s="13" t="n">
-        <v>32</v>
-      </c>
-      <c r="N8" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="O8" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="P8" s="13" t="n">
-        <v>21</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
-        <v>269</v>
-      </c>
-      <c r="C9" s="15" t="n">
+      <c r="B9" s="13" t="n">
         <v>311</v>
       </c>
-      <c r="D9" s="15" t="n">
-        <v>343</v>
+      <c r="C9" s="13" t="n">
+        <v>363</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="A1:P1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1095,40 +982,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y9"/>
+  <dimension ref="A1:Q9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="7" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="7" customWidth="1" min="6" max="6"/>
-    <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="7" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
-    <col width="7" customWidth="1" min="12" max="12"/>
-    <col width="7" customWidth="1" min="13" max="13"/>
-    <col width="7" customWidth="1" min="14" max="14"/>
-    <col width="7" customWidth="1" min="15" max="15"/>
-    <col width="7" customWidth="1" min="16" max="16"/>
-    <col width="7" customWidth="1" min="17" max="17"/>
-    <col width="7" customWidth="1" min="18" max="18"/>
-    <col width="7" customWidth="1" min="19" max="19"/>
-    <col width="7" customWidth="1" min="20" max="20"/>
-    <col width="7" customWidth="1" min="21" max="21"/>
-    <col width="7" customWidth="1" min="22" max="22"/>
-    <col width="7" customWidth="1" min="23" max="23"/>
-    <col width="7" customWidth="1" min="24" max="24"/>
-    <col width="7" customWidth="1" min="25" max="25"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="8" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="8" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t>CANTIDADES POR COLORES — RANGO DE ACCIÓN</t>
+          <t>CANTIDADES POR COLORES — MÍNIMO Y MÁXIMO</t>
         </is>
       </c>
     </row>
@@ -1143,37 +1022,37 @@
           <t>1</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
+      <c r="F2" s="5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
       <c r="H2" s="5" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr">
-        <is>
           <t>6</t>
         </is>
       </c>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr">
-        <is>
           <t>12</t>
         </is>
       </c>
-      <c r="W2" s="5" t="inlineStr">
+      <c r="P2" s="5" t="inlineStr">
         <is>
           <t>14</t>
         </is>
@@ -1187,29 +1066,29 @@
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="D3" s="8" t="inlineStr">
-        <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="E3" s="6" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
       <c r="H3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
@@ -1217,29 +1096,29 @@
       </c>
       <c r="I3" s="7" t="inlineStr">
         <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="K3" s="6" t="inlineStr">
+      <c r="J3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Mín</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="inlineStr">
+        <is>
+          <t>Máx</t>
+        </is>
+      </c>
       <c r="N3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
@@ -1247,302 +1126,199 @@
       </c>
       <c r="O3" s="7" t="inlineStr">
         <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="Q3" s="6" t="inlineStr">
+      <c r="P3" s="6" t="inlineStr">
         <is>
           <t>Mín</t>
         </is>
       </c>
-      <c r="R3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
+      <c r="Q3" s="7" t="inlineStr">
         <is>
           <t>Máx</t>
         </is>
       </c>
-      <c r="T3" s="6" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="U3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="V3" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
-      <c r="W3" s="6" t="inlineStr">
-        <is>
-          <t>Mín</t>
-        </is>
-      </c>
-      <c r="X3" s="7" t="inlineStr">
-        <is>
-          <t>Sol</t>
-        </is>
-      </c>
-      <c r="Y3" s="8" t="inlineStr">
-        <is>
-          <t>Máx</t>
-        </is>
-      </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="inlineStr">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>Playuela</t>
         </is>
       </c>
-      <c r="B4" s="10" t="n"/>
-      <c r="C4" s="11" t="n"/>
-      <c r="D4" s="12" t="n"/>
+      <c r="B4" s="9" t="n"/>
+      <c r="C4" s="10" t="n"/>
+      <c r="D4" s="9" t="n"/>
       <c r="E4" s="10" t="n"/>
-      <c r="F4" s="11" t="n"/>
-      <c r="G4" s="12" t="n"/>
-      <c r="H4" s="10" t="n"/>
-      <c r="I4" s="11" t="n"/>
-      <c r="J4" s="12" t="n"/>
+      <c r="F4" s="9" t="n"/>
+      <c r="G4" s="10" t="n"/>
+      <c r="H4" s="9" t="n"/>
+      <c r="I4" s="10" t="n"/>
+      <c r="J4" s="9" t="n"/>
       <c r="K4" s="10" t="n"/>
-      <c r="L4" s="11" t="n"/>
-      <c r="M4" s="12" t="n"/>
-      <c r="N4" s="10" t="n"/>
-      <c r="O4" s="11" t="n"/>
-      <c r="P4" s="12" t="n"/>
-      <c r="Q4" s="13" t="n">
+      <c r="L4" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="R4" s="13" t="n">
+      <c r="M4" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="S4" s="13" t="n">
+      <c r="N4" s="9" t="n"/>
+      <c r="O4" s="10" t="n"/>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="10" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Sal</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="10" t="n"/>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="10" t="n"/>
+      <c r="P5" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q5" s="11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Tucupido</t>
+        </is>
+      </c>
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="9" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="9" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="9" t="n"/>
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="9" t="n"/>
+      <c r="M6" s="10" t="n"/>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="10" t="n"/>
+      <c r="P6" s="9" t="n"/>
+      <c r="Q6" s="10" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Sombrero</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n"/>
+      <c r="C7" s="10" t="n"/>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="10" t="n"/>
+      <c r="F7" s="9" t="n"/>
+      <c r="G7" s="10" t="n"/>
+      <c r="H7" s="9" t="n"/>
+      <c r="I7" s="10" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="10" t="n"/>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="10" t="n"/>
+      <c r="N7" s="9" t="n"/>
+      <c r="O7" s="10" t="n"/>
+      <c r="P7" s="9" t="n"/>
+      <c r="Q7" s="10" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Nuevo color (lanzamiento)</t>
+        </is>
+      </c>
+      <c r="B8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="T4" s="10" t="n"/>
-      <c r="U4" s="11" t="n"/>
-      <c r="V4" s="12" t="n"/>
-      <c r="W4" s="10" t="n"/>
-      <c r="X4" s="11" t="n"/>
-      <c r="Y4" s="12" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="9" t="inlineStr">
-        <is>
-          <t>Sal</t>
-        </is>
-      </c>
-      <c r="B5" s="10" t="n"/>
-      <c r="C5" s="11" t="n"/>
-      <c r="D5" s="12" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="11" t="n"/>
-      <c r="G5" s="12" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="11" t="n"/>
-      <c r="J5" s="12" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="11" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="11" t="n"/>
-      <c r="P5" s="12" t="n"/>
-      <c r="Q5" s="10" t="n"/>
-      <c r="R5" s="11" t="n"/>
-      <c r="S5" s="12" t="n"/>
-      <c r="T5" s="10" t="n"/>
-      <c r="U5" s="11" t="n"/>
-      <c r="V5" s="12" t="n"/>
-      <c r="W5" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="X5" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y5" s="13" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="9" t="inlineStr">
-        <is>
-          <t>Tucupido</t>
-        </is>
-      </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="11" t="n"/>
-      <c r="D6" s="12" t="n"/>
-      <c r="E6" s="10" t="n"/>
-      <c r="F6" s="11" t="n"/>
-      <c r="G6" s="12" t="n"/>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="11" t="n"/>
-      <c r="J6" s="12" t="n"/>
-      <c r="K6" s="10" t="n"/>
-      <c r="L6" s="11" t="n"/>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="10" t="n"/>
-      <c r="O6" s="11" t="n"/>
-      <c r="P6" s="12" t="n"/>
-      <c r="Q6" s="10" t="n"/>
-      <c r="R6" s="11" t="n"/>
-      <c r="S6" s="12" t="n"/>
-      <c r="T6" s="10" t="n"/>
-      <c r="U6" s="11" t="n"/>
-      <c r="V6" s="12" t="n"/>
-      <c r="W6" s="10" t="n"/>
-      <c r="X6" s="11" t="n"/>
-      <c r="Y6" s="12" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>Sombrero</t>
-        </is>
-      </c>
-      <c r="B7" s="10" t="n"/>
-      <c r="C7" s="11" t="n"/>
-      <c r="D7" s="12" t="n"/>
-      <c r="E7" s="10" t="n"/>
-      <c r="F7" s="11" t="n"/>
-      <c r="G7" s="12" t="n"/>
-      <c r="H7" s="10" t="n"/>
-      <c r="I7" s="11" t="n"/>
-      <c r="J7" s="12" t="n"/>
-      <c r="K7" s="10" t="n"/>
-      <c r="L7" s="11" t="n"/>
-      <c r="M7" s="12" t="n"/>
-      <c r="N7" s="10" t="n"/>
-      <c r="O7" s="11" t="n"/>
-      <c r="P7" s="12" t="n"/>
-      <c r="Q7" s="10" t="n"/>
-      <c r="R7" s="11" t="n"/>
-      <c r="S7" s="12" t="n"/>
-      <c r="T7" s="10" t="n"/>
-      <c r="U7" s="11" t="n"/>
-      <c r="V7" s="12" t="n"/>
-      <c r="W7" s="10" t="n"/>
-      <c r="X7" s="11" t="n"/>
-      <c r="Y7" s="12" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>Nuevo color (lanzamiento)</t>
-        </is>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="13" t="n">
+      <c r="D8" s="11" t="n">
+        <v>7</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="G8" s="13" t="n">
+      <c r="H8" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="H8" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="I8" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="J8" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="L8" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="M8" s="13" t="n">
+      <c r="I8" s="11" t="n">
+        <v>10</v>
+      </c>
+      <c r="J8" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="N8" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="O8" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="P8" s="13" t="n">
+      <c r="K8" s="11" t="n">
+        <v>11</v>
+      </c>
+      <c r="L8" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="Q8" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="R8" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="S8" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="T8" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="U8" s="13" t="n">
+      <c r="M8" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="N8" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="V8" s="13" t="n">
+      <c r="O8" s="11" t="n">
+        <v>16</v>
+      </c>
+      <c r="P8" s="11" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q8" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="W8" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="X8" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="Y8" s="13" t="n">
-        <v>13</v>
-      </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
-        <v>58</v>
-      </c>
-      <c r="C9" s="15" t="n">
+      <c r="B9" s="13" t="n">
         <v>70</v>
       </c>
-      <c r="D9" s="15" t="n">
-        <v>76</v>
+      <c r="C9" s="13" t="n">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="T2:V2"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="K2:M2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="A1:Y1"/>
-    <mergeCell ref="H2:J2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="W2:Y2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="P2:Q2"/>
+    <mergeCell ref="A1:Q1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1554,16 +1330,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A31"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="95" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="16" t="inlineStr">
-        <is>
-          <t>METODOLOGÍA — RANGO DE ACCIÓN SHORT PLAYA SUBLIMADO</t>
+      <c r="A1" s="14" t="inlineStr">
+        <is>
+          <t>METODOLOGÍA — MÍNIMO Y MÁXIMO SHORT PLAYA SUBLIMADO</t>
         </is>
       </c>
     </row>
@@ -1571,189 +1347,137 @@
       <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="16" t="inlineStr">
-        <is>
-          <t>1. SOLICITADO (referencia del dashboard)</t>
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>1. MÍNIMO (compromiso de producción)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Cantidad por color/talla según rotación ajustada × factor temporada alta (×1.4).</t>
+          <t xml:space="preserve">   Son las cantidades establecidas en el dashboard por color y talla.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Rotación base: promedio últimos 6 meses completos, con diciembre ponderado ×1.4.</t>
+          <t xml:space="preserve">   Representan lo que SÍ hay que fabricar sí o sí: curva óptima, cobertura 3 meses,</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Cobertura objetivo: 3 meses (lead time 90 días).</t>
+          <t xml:space="preserve">   factor temporada alta (×{hs}), diciembre ponderado, tiendas nuevas (VELA, Barquisimeto)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Color nuevo: benchmark top 3 colores (Sal, Playuela, Tucupido) × participación de red</t>
+          <t xml:space="preserve">   y color de lanzamiento.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   incluyendo VELA (1.5× GRIETA) y Barquisimeto, con ramp-up 70% en apertura.</t>
-        </is>
-      </c>
+      <c r="A8" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>2. MÁXIMO (rango de acción hacia arriba)</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
-        <is>
-          <t>2. MÍNIMO (piso — producción no debería bajar de aquí)</t>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Si hay tela disponible que hoy está parada, producción puede subir HASTA el máximo.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">   CAB tallas M/L/XL: 90% del solicitado.</t>
+          <t xml:space="preserve">   El techo es el menor entre:</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">   CAB tallas S/2XL: 70% del solicitado.</t>
+          <t xml:space="preserve">   a) Mínimo + 15% (20% en color de lanzamiento)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">   KIDS tallas 6–14: 85% del solicitado.</t>
+          <t xml:space="preserve">   b) Unidades para no superar 6 meses de cobertura por talla (anti sobrestock).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   KIDS tallas 1–4: 70% del solicitado.</t>
-        </is>
-      </c>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Si solicitado = 0 → mínimo = 0.</t>
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>3. LÓGICA DE LA REUNIÓN</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • El mínimo cubre disponibilidad en red (diciembre, enero, carnaval).</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>3. MÁXIMO (techo — anti sobrestock)</t>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   • El máximo permite aprovechar tela adicional sin dejarla idle ni inflar inventario.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Menor valor entre:</t>
+          <t xml:space="preserve">   • Producción decide cuánto fabricar entre Mín y Máx según tela y capacidad del mes.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   a) Solicitado + 10%</t>
+          <t xml:space="preserve">   • Lo fabricado se distribuye y mueve entre tiendas para cubrir huecos.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   b) Unidades para no superar 6 meses de cobertura (stock actual + producción).</t>
-        </is>
-      </c>
+      <c r="A20" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   El máximo nunca es menor que el solicitado.</t>
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>4. EJEMPLO</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr"/>
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Si Mín = 41 und talla M color nuevo y Máx = 47 und → hay 6 und de margen</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>4. CONTEXTO TEMPORADA Y TIENDAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Proyección orientada a picos: diciembre, enero y carnaval (factor temporada alta).</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Uso inteligente de tela disponible: fabricar según rango y redistribuir entre tiendas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Tiendas nuevas absorben parte del volumen de lanzamiento sin sobrecargar stock en una sola tienda.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>5. CÓMO USA PRODUCCIÓN EL RANGO</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Fabricar preferentemente en el SOLICITADO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Si hay restricción de tela/capacidad: no bajar del MÍNIMO en tallas núcleo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   • Si hay tela adicional y demanda confirma pico festivo: puede subir hasta el MÁXIMO sin aprobación extra.</t>
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   para usar tela extra si el pico festivo lo justifica.</t>
         </is>
       </c>
     </row>

</xml_diff>